<commit_message>
feat(analysis): add bootstrapped effect size pipeline and custom forest plots
- Extracted and modularized effect size calculations into `bootstrap_effect_sizes.m` to compute Cohen's dz and 95% bootstrapped CIs for both scalar variables and trajectory time windows.
- Created `plot_and_save_effect_sizes.m` to generate horizontal forest plots per analysis flavor and a cross-flavor difference comparison figure vs. Keyboard RT (with shaded flavor blocks, category headers, and right-aligned labels).
- Integrated effect size bootstrapping and visualization into `RUN_ME.m`.
</commit_message>
<xml_diff>
--- a/analysis/statistics/All_Statistics.xlsx
+++ b/analysis/statistics/All_Statistics.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="110" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="661" uniqueCount="76">
   <si>
     <t>name</t>
   </si>
@@ -244,6 +244,9 @@
   </si>
   <si>
     <t>reach_CI_high</t>
+  </si>
+  <si>
+    <t>---- vel --------</t>
   </si>
 </sst>
 </file>
@@ -292,25 +295,25 @@
   <dimension ref="A1:S9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="true"/>
-    <col min="2" max="2" width="26.6640625" customWidth="true"/>
-    <col min="3" max="3" width="26.6640625" customWidth="true"/>
-    <col min="4" max="4" width="19.6640625" customWidth="true"/>
-    <col min="5" max="5" width="29.77734375" customWidth="true"/>
-    <col min="6" max="6" width="13.5546875" customWidth="true"/>
-    <col min="7" max="7" width="13.5546875" customWidth="true"/>
-    <col min="8" max="8" width="13.5546875" customWidth="true"/>
-    <col min="9" max="9" width="13.5546875" customWidth="true"/>
-    <col min="10" max="10" width="15.21875" customWidth="true"/>
-    <col min="11" max="11" width="12.21875" customWidth="true"/>
-    <col min="12" max="12" width="15.5546875" customWidth="true"/>
-    <col min="13" max="13" width="13.21875" customWidth="true"/>
-    <col min="14" max="14" width="14.33203125" customWidth="true"/>
-    <col min="15" max="15" width="3" customWidth="true"/>
-    <col min="16" max="16" width="14.21875" customWidth="true"/>
-    <col min="17" max="17" width="15.21875" customWidth="true"/>
-    <col min="18" max="18" width="14.5546875" customWidth="true"/>
-    <col min="19" max="19" width="21.6640625" customWidth="true"/>
+    <col min="1" max="1" width="33.5703125" customWidth="true"/>
+    <col min="2" max="2" width="28.85546875" customWidth="true"/>
+    <col min="3" max="3" width="28.85546875" customWidth="true"/>
+    <col min="4" max="4" width="21.28515625" customWidth="true"/>
+    <col min="5" max="5" width="32.5703125" customWidth="true"/>
+    <col min="6" max="6" width="13.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13.7109375" customWidth="true"/>
+    <col min="8" max="8" width="13.7109375" customWidth="true"/>
+    <col min="9" max="9" width="13.7109375" customWidth="true"/>
+    <col min="10" max="10" width="15.42578125" customWidth="true"/>
+    <col min="11" max="11" width="12.42578125" customWidth="true"/>
+    <col min="12" max="12" width="15.7109375" customWidth="true"/>
+    <col min="13" max="13" width="13.42578125" customWidth="true"/>
+    <col min="14" max="14" width="15.85546875" customWidth="true"/>
+    <col min="15" max="15" width="3.140625" customWidth="true"/>
+    <col min="16" max="16" width="14.42578125" customWidth="true"/>
+    <col min="17" max="17" width="15.42578125" customWidth="true"/>
+    <col min="18" max="18" width="14.7109375" customWidth="true"/>
+    <col min="19" max="19" width="23.28515625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -850,18 +853,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.109375" customWidth="true"/>
-    <col min="2" max="2" width="6.44140625" customWidth="true"/>
-    <col min="3" max="3" width="9.44140625" customWidth="true"/>
-    <col min="4" max="4" width="8.6640625" customWidth="true"/>
-    <col min="5" max="5" width="11.5546875" customWidth="true"/>
-    <col min="6" max="6" width="14.5546875" customWidth="true"/>
-    <col min="7" max="7" width="12.5546875" customWidth="true"/>
-    <col min="8" max="8" width="11.5546875" customWidth="true"/>
-    <col min="9" max="9" width="21.6640625" customWidth="true"/>
+    <col min="1" max="1" width="20.85546875" customWidth="true"/>
+    <col min="2" max="2" width="7.140625" customWidth="true"/>
+    <col min="3" max="3" width="10.28515625" customWidth="true"/>
+    <col min="4" max="4" width="9.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="14.7109375" customWidth="true"/>
+    <col min="7" max="7" width="12.7109375" customWidth="true"/>
+    <col min="8" max="8" width="11.7109375" customWidth="true"/>
+    <col min="9" max="9" width="23.28515625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -910,16 +913,16 @@
         <v>62.678170577696179</v>
       </c>
       <c r="F2" s="0">
-        <v>0.033002989742891953</v>
+        <v>0.032792132688099773</v>
       </c>
       <c r="G2" s="0">
         <v>0.71521349767835019</v>
       </c>
       <c r="H2" s="0">
-        <v>3.6167126446069036</v>
+        <v>3.6208511701072754</v>
       </c>
       <c r="I2" s="0">
-        <v>0.039603587691470342</v>
+        <v>0.039350559225719728</v>
       </c>
     </row>
     <row r="3">
@@ -939,16 +942,16 @@
         <v>78.217592804323957</v>
       </c>
       <c r="F3" s="0">
-        <v>0.0020315800748353929</v>
+        <v>0.0023466671439258402</v>
       </c>
       <c r="G3" s="0">
         <v>0.71402566621136665</v>
       </c>
       <c r="H3" s="0">
-        <v>6.0282372576687315</v>
+        <v>5.8743426044913081</v>
       </c>
       <c r="I3" s="0">
-        <v>0.0020315800748353929</v>
+        <v>0.0023466671439258402</v>
       </c>
     </row>
     <row r="4">
@@ -968,16 +971,45 @@
         <v>60.218858391558385</v>
       </c>
       <c r="F4" s="0">
-        <v>0.0018910700747309939</v>
+        <v>0.0016522187376124542</v>
       </c>
       <c r="G4" s="0">
         <v>0.64672994369148595</v>
       </c>
       <c r="H4" s="0">
-        <v>6.3364669217956298</v>
+        <v>6.2029429243702685</v>
       </c>
       <c r="I4" s="0">
-        <v>0.0037821401494619877</v>
+        <v>0.0033044374752249084</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="0">
+        <v>1</v>
+      </c>
+      <c r="C5" s="0">
+        <v>15</v>
+      </c>
+      <c r="D5" s="0">
+        <v>30</v>
+      </c>
+      <c r="E5" s="0">
+        <v>65.045480487551046</v>
+      </c>
+      <c r="F5" s="0">
+        <v>0.0017306036164095318</v>
+      </c>
+      <c r="G5" s="0">
+        <v>0.74222660264153839</v>
+      </c>
+      <c r="H5" s="0">
+        <v>6.0310488443850261</v>
+      </c>
+      <c r="I5" s="0">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -989,20 +1021,20 @@
   <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="true"/>
-    <col min="2" max="2" width="11.5546875" customWidth="true"/>
-    <col min="3" max="3" width="7.21875" customWidth="true"/>
-    <col min="4" max="4" width="4.6640625" customWidth="true"/>
-    <col min="5" max="5" width="9" customWidth="true"/>
-    <col min="6" max="6" width="12.44140625" customWidth="true"/>
-    <col min="7" max="7" width="12.109375" customWidth="true"/>
-    <col min="8" max="8" width="7.5546875" customWidth="true"/>
-    <col min="9" max="9" width="11.44140625" customWidth="true"/>
-    <col min="10" max="10" width="15.88671875" customWidth="true"/>
-    <col min="11" max="11" width="8.44140625" customWidth="true"/>
-    <col min="12" max="12" width="8.33203125" customWidth="true"/>
-    <col min="13" max="13" width="4.109375" customWidth="true"/>
-    <col min="14" max="14" width="3.88671875" customWidth="true"/>
+    <col min="1" max="1" width="12.7109375" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="8.140625" customWidth="true"/>
+    <col min="4" max="4" width="5.140625" customWidth="true"/>
+    <col min="5" max="5" width="9.7109375" customWidth="true"/>
+    <col min="6" max="6" width="13.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13.28515625" customWidth="true"/>
+    <col min="8" max="8" width="8.28515625" customWidth="true"/>
+    <col min="9" max="9" width="12.5703125" customWidth="true"/>
+    <col min="10" max="10" width="17.42578125" customWidth="true"/>
+    <col min="11" max="11" width="9.28515625" customWidth="true"/>
+    <col min="12" max="12" width="9" customWidth="true"/>
+    <col min="13" max="13" width="4.7109375" customWidth="true"/>
+    <col min="14" max="14" width="4.28515625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2378,20 +2410,20 @@
   <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="true"/>
-    <col min="2" max="2" width="11.5546875" customWidth="true"/>
-    <col min="3" max="3" width="7.21875" customWidth="true"/>
-    <col min="4" max="4" width="4.6640625" customWidth="true"/>
-    <col min="5" max="5" width="9" customWidth="true"/>
-    <col min="6" max="6" width="12.44140625" customWidth="true"/>
-    <col min="7" max="7" width="12.109375" customWidth="true"/>
-    <col min="8" max="8" width="7.5546875" customWidth="true"/>
-    <col min="9" max="9" width="11.44140625" customWidth="true"/>
-    <col min="10" max="10" width="15.88671875" customWidth="true"/>
-    <col min="11" max="11" width="8.44140625" customWidth="true"/>
-    <col min="12" max="12" width="8.33203125" customWidth="true"/>
-    <col min="13" max="13" width="4.109375" customWidth="true"/>
-    <col min="14" max="14" width="4" customWidth="true"/>
+    <col min="1" max="1" width="12.7109375" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" customWidth="true"/>
+    <col min="3" max="3" width="8.140625" customWidth="true"/>
+    <col min="4" max="4" width="5.140625" customWidth="true"/>
+    <col min="5" max="5" width="9.7109375" customWidth="true"/>
+    <col min="6" max="6" width="13.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13.28515625" customWidth="true"/>
+    <col min="8" max="8" width="8.28515625" customWidth="true"/>
+    <col min="9" max="9" width="12.5703125" customWidth="true"/>
+    <col min="10" max="10" width="17.42578125" customWidth="true"/>
+    <col min="11" max="11" width="9.28515625" customWidth="true"/>
+    <col min="12" max="12" width="9" customWidth="true"/>
+    <col min="13" max="13" width="4.7109375" customWidth="true"/>
+    <col min="14" max="14" width="4.28515625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3767,11 +3799,11 @@
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" customWidth="true"/>
-    <col min="2" max="2" width="13.21875" customWidth="true"/>
-    <col min="3" max="3" width="13.21875" customWidth="true"/>
-    <col min="4" max="4" width="13.21875" customWidth="true"/>
-    <col min="5" max="5" width="13.21875" customWidth="true"/>
+    <col min="1" max="1" width="10.7109375" customWidth="true"/>
+    <col min="2" max="2" width="14.42578125" customWidth="true"/>
+    <col min="3" max="3" width="14.42578125" customWidth="true"/>
+    <col min="4" max="4" width="14.42578125" customWidth="true"/>
+    <col min="5" max="5" width="14.42578125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4310,11 +4342,11 @@
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" customWidth="true"/>
-    <col min="2" max="2" width="13.21875" customWidth="true"/>
-    <col min="3" max="3" width="13.21875" customWidth="true"/>
-    <col min="4" max="4" width="13.21875" customWidth="true"/>
-    <col min="5" max="5" width="13.21875" customWidth="true"/>
+    <col min="1" max="1" width="10.7109375" customWidth="true"/>
+    <col min="2" max="2" width="14.42578125" customWidth="true"/>
+    <col min="3" max="3" width="14.42578125" customWidth="true"/>
+    <col min="4" max="4" width="14.42578125" customWidth="true"/>
+    <col min="5" max="5" width="14.42578125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4853,21 +4885,21 @@
   <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" customWidth="true"/>
-    <col min="2" max="2" width="11.5546875" customWidth="true"/>
-    <col min="3" max="3" width="10.5546875" customWidth="true"/>
-    <col min="4" max="4" width="11.5546875" customWidth="true"/>
-    <col min="5" max="5" width="11.5546875" customWidth="true"/>
-    <col min="6" max="6" width="11.5546875" customWidth="true"/>
-    <col min="7" max="7" width="5.5546875" customWidth="true"/>
-    <col min="8" max="8" width="12.5546875" customWidth="true"/>
-    <col min="9" max="9" width="11.5546875" customWidth="true"/>
-    <col min="10" max="10" width="10.5546875" customWidth="true"/>
-    <col min="11" max="11" width="11.5546875" customWidth="true"/>
-    <col min="12" max="12" width="8.21875" customWidth="true"/>
-    <col min="13" max="13" width="11.5546875" customWidth="true"/>
-    <col min="14" max="14" width="12.21875" customWidth="true"/>
-    <col min="15" max="15" width="12.5546875" customWidth="true"/>
+    <col min="1" max="1" width="10.28515625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="10.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+    <col min="7" max="7" width="6.140625" customWidth="true"/>
+    <col min="8" max="8" width="12.7109375" customWidth="true"/>
+    <col min="9" max="9" width="11.7109375" customWidth="true"/>
+    <col min="10" max="10" width="10.85546875" customWidth="true"/>
+    <col min="11" max="11" width="11.7109375" customWidth="true"/>
+    <col min="12" max="12" width="8.85546875" customWidth="true"/>
+    <col min="13" max="13" width="11.7109375" customWidth="true"/>
+    <col min="14" max="14" width="13" customWidth="true"/>
+    <col min="15" max="15" width="13.5703125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>